<commit_message>
Updating Test Scenarios (Final)
</commit_message>
<xml_diff>
--- a/03-Test_Scenarios/01-Test_Scenarios.xlsx
+++ b/03-Test_Scenarios/01-Test_Scenarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my things\SQA projects\QADemo E-Commerce Application Manual Testing\QADemoE-CommerceApplicationManualTesting\03-Test_Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3280355-3E25-4A03-A25A-07C84EE994A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C983D4CF-9C12-47D5-AC81-52D095794AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="216">
   <si>
     <t>Scenario ID</t>
   </si>
@@ -213,15 +213,6 @@
     <t>TS-046</t>
   </si>
   <si>
-    <t>TS-047</t>
-  </si>
-  <si>
-    <t>Order Details Review</t>
-  </si>
-  <si>
-    <t>TS-048</t>
-  </si>
-  <si>
     <t>FR-011</t>
   </si>
   <si>
@@ -252,9 +243,6 @@
     <t>Compatibility</t>
   </si>
   <si>
-    <t>Responsive</t>
-  </si>
-  <si>
     <t>NFR-001</t>
   </si>
   <si>
@@ -267,9 +255,6 @@
     <t>Performance</t>
   </si>
   <si>
-    <t>—</t>
-  </si>
-  <si>
     <t>Regression</t>
   </si>
   <si>
@@ -339,9 +324,6 @@
     <t>Product Display</t>
   </si>
   <si>
-    <t>Product Category Browsing</t>
-  </si>
-  <si>
     <t>Product Search</t>
   </si>
   <si>
@@ -420,12 +402,6 @@
     <t>Verify that product prices remain consistent from product details through checkout</t>
   </si>
   <si>
-    <t>Cart to Checkout</t>
-  </si>
-  <si>
-    <t>Verify that customers can successfully proceed from the cart to checkout</t>
-  </si>
-  <si>
     <t>Incomplete Order Placement</t>
   </si>
   <si>
@@ -441,81 +417,21 @@
     <t>Verify that order confirmation displays the relevant order information correctly</t>
   </si>
   <si>
-    <t>Order Identifier</t>
-  </si>
-  <si>
-    <t>Verify that a unique order identifier is generated for each successful order</t>
-  </si>
-  <si>
-    <t>Order Details Access</t>
-  </si>
-  <si>
-    <t>Verify that customers can access the details of their placed orders</t>
-  </si>
-  <si>
-    <t>Order Details Information</t>
-  </si>
-  <si>
-    <t>Verify that order details display accurate products, quantities, prices and total</t>
-  </si>
-  <si>
-    <t>Order Status</t>
-  </si>
-  <si>
-    <t>Verify that customers can view the current status of their orders</t>
-  </si>
-  <si>
-    <t>Order Information Consistency</t>
-  </si>
-  <si>
-    <t>Verify that order information remains consistent between confirmation and order details</t>
-  </si>
-  <si>
     <t>Customer Input Validation</t>
   </si>
   <si>
-    <t>Verify that applicable customer-facing forms validate input correctly</t>
-  </si>
-  <si>
-    <t>Session Security</t>
-  </si>
-  <si>
     <t>Verify that customer sessions prevent unauthorized access to protected information</t>
   </si>
   <si>
-    <t>Order Data Integrity</t>
-  </si>
-  <si>
-    <t>Verify that product, cart, checkout and order prices remain accurate throughout the order process</t>
-  </si>
-  <si>
     <t>Error Handling</t>
   </si>
   <si>
     <t>Verify that the application handles failed operations with appropriate feedback</t>
   </si>
   <si>
-    <t>Browser and Device Compatibility</t>
-  </si>
-  <si>
-    <t>Verify that core customer workflows function correctly across supported browsers and devices</t>
-  </si>
-  <si>
-    <t>Responsive Design</t>
-  </si>
-  <si>
-    <t>Verify that customer-facing pages remain usable across supported screen sizes</t>
-  </si>
-  <si>
     <t>Verify that customers can complete the main shopping journey clearly and easily</t>
   </si>
   <si>
-    <t>Application Performance</t>
-  </si>
-  <si>
-    <t>Verify that key customer-facing pages and operations respond within acceptable time</t>
-  </si>
-  <si>
     <t>API Response Validation</t>
   </si>
   <si>
@@ -546,18 +462,6 @@
     <t>Verify that order and status information remains consistent between the application and database</t>
   </si>
   <si>
-    <t>Regression Testing</t>
-  </si>
-  <si>
-    <t>Verify that existing customer workflows continue to function correctly after system changes</t>
-  </si>
-  <si>
-    <t>End-to-End Purchase Flow</t>
-  </si>
-  <si>
-    <t>Verify that the complete customer journey works successfully from login through order details and status</t>
-  </si>
-  <si>
     <t>FR-001</t>
   </si>
   <si>
@@ -621,9 +525,6 @@
     <t xml:space="preserve">Security </t>
   </si>
   <si>
-    <t>Verify that selecting an available category displays products belonging to that category</t>
-  </si>
-  <si>
     <t>Positive / Data Validation</t>
   </si>
   <si>
@@ -667,6 +568,111 @@
   </si>
   <si>
     <t>Search Product</t>
+  </si>
+  <si>
+    <t>Successful Order Confirmation</t>
+  </si>
+  <si>
+    <t>Order Information and Status</t>
+  </si>
+  <si>
+    <t>View Placed Orders</t>
+  </si>
+  <si>
+    <t>View Unique Order IDs</t>
+  </si>
+  <si>
+    <t>Verify Delivery Information</t>
+  </si>
+  <si>
+    <t>View Current Order Status</t>
+  </si>
+  <si>
+    <t>Placed Order Details</t>
+  </si>
+  <si>
+    <t>Verify each placed order displays its corresponding unique order ID</t>
+  </si>
+  <si>
+    <t>Verify that the relevant product, quantity and price are displayed correctly in the order information</t>
+  </si>
+  <si>
+    <t>Data Consistency</t>
+  </si>
+  <si>
+    <t>Verify that the order details display the delivery information entered during checkout</t>
+  </si>
+  <si>
+    <t>Verify that the order details display the current applicable status and reflect status changes when available</t>
+  </si>
+  <si>
+    <t>State Transition / Data Validation</t>
+  </si>
+  <si>
+    <t>Shopping Journey Usability</t>
+  </si>
+  <si>
+    <t>Page Response Times</t>
+  </si>
+  <si>
+    <t>Session Authorization</t>
+  </si>
+  <si>
+    <t>Failed Operation Feedback</t>
+  </si>
+  <si>
+    <t>Verify that core customer workflows function correctly across supported browsers</t>
+  </si>
+  <si>
+    <t>Cross-Browser</t>
+  </si>
+  <si>
+    <t>Cross-Device</t>
+  </si>
+  <si>
+    <t>Browser Compatibility</t>
+  </si>
+  <si>
+    <t>Device Compatibility</t>
+  </si>
+  <si>
+    <t>Verify that customer-facing pages remain usable across supported devices or screen sizes</t>
+  </si>
+  <si>
+    <t>Verify that the product listing displays the available products with the relevant product information</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Verify that the product prices, quantities and order total recorded for a placed order are consistent with the confirmed order details</t>
+  </si>
+  <si>
+    <t>Order Price Data Integrity</t>
+  </si>
+  <si>
+    <t>End-to-End Customer Purchase Journey</t>
+  </si>
+  <si>
+    <t>Verify that a customer can complete the end-to-end shopping journey, from login and product discovery through cart management, checkout, order placement, confirmation and order details review</t>
+  </si>
+  <si>
+    <t>Customer Workflow Regression Testing</t>
+  </si>
+  <si>
+    <t>Verify that previously working critical customer workflows continue to function as expected after application changes</t>
+  </si>
+  <si>
+    <t>Verify that key customer-facing pages and operations meet the response-time targets defined in the Test Strategy under the specified test conditions</t>
+  </si>
+  <si>
+    <t>Verify that all applicable customer-facing forms validate input correctly</t>
+  </si>
+  <si>
+    <t>Verify customers can access their placed orders and multiple orders are distinguishable</t>
+  </si>
+  <si>
+    <t>Cross-functional</t>
   </si>
 </sst>
 </file>
@@ -889,8 +895,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1059436E-1C1B-4B5F-B920-6AA0420AD722}" name="Table3" displayName="Table3" ref="A13:G61" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A13:G61" xr:uid="{1059436E-1C1B-4B5F-B920-6AA0420AD722}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1059436E-1C1B-4B5F-B920-6AA0420AD722}" name="Table3" displayName="Table3" ref="A13:G59" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A13:G59" xr:uid="{1059436E-1C1B-4B5F-B920-6AA0420AD722}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{2543D124-61AE-419E-A477-5339FBB9DB8D}" name="Scenario ID" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{F1185ACC-CC8E-4BF8-AB59-6CFF78CBC5AA}" name="Test Scenario" dataDxfId="5"/>
@@ -1167,66 +1173,66 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:G61"/>
+  <dimension ref="A2:G59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="29.88671875" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="45" customWidth="1"/>
-    <col min="6" max="6" width="23.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="2" max="2" width="30.77734375" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="45.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.33203125" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" customWidth="1"/>
     <col min="8" max="8" width="14.109375" customWidth="1"/>
     <col min="9" max="9" width="14.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>187</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -1237,7 +1243,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>188</v>
+        <v>156</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>2</v>
@@ -1246,7 +1252,7 @@
         <v>3</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>191</v>
+        <v>159</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>4</v>
@@ -1257,19 +1263,19 @@
         <v>5</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>190</v>
+        <v>158</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>7</v>
@@ -1280,19 +1286,19 @@
         <v>8</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>195</v>
+        <v>163</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>193</v>
+        <v>161</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>194</v>
+        <v>162</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>7</v>
@@ -1303,19 +1309,19 @@
         <v>10</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>196</v>
+        <v>164</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>9</v>
@@ -1326,19 +1332,19 @@
         <v>11</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>197</v>
+        <v>165</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>13</v>
@@ -1349,19 +1355,19 @@
         <v>12</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>9</v>
@@ -1372,19 +1378,19 @@
         <v>14</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>9</v>
@@ -1395,19 +1401,19 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>7</v>
@@ -1417,43 +1423,43 @@
       <c r="A21" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>104</v>
+      <c r="B21" s="7" t="s">
+        <v>180</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>178</v>
+        <v>154</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>18</v>
+        <v>99</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>198</v>
+        <v>100</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>213</v>
+      <c r="B22" s="1" t="s">
+        <v>101</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>186</v>
+        <v>147</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>105</v>
+        <v>26</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>192</v>
+        <v>166</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>9</v>
@@ -1464,19 +1470,19 @@
         <v>19</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>179</v>
+        <v>147</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>26</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>199</v>
+        <v>167</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>9</v>
@@ -1487,22 +1493,22 @@
         <v>20</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>179</v>
+        <v>148</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1510,22 +1516,22 @@
         <v>21</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>31</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1533,19 +1539,19 @@
         <v>22</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>31</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>9</v>
@@ -1556,22 +1562,22 @@
         <v>23</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>31</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>192</v>
+        <v>166</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1579,22 +1585,22 @@
         <v>24</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>31</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>199</v>
+        <v>166</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1602,19 +1608,19 @@
         <v>25</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>31</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>201</v>
+        <v>160</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>9</v>
@@ -1625,22 +1631,22 @@
         <v>27</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>31</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1648,65 +1654,65 @@
         <v>28</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>180</v>
+        <v>149</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>181</v>
+        <v>149</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>40</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>201</v>
+        <v>168</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>181</v>
+        <v>149</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>40</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>201</v>
+        <v>169</v>
       </c>
       <c r="G33" s="1" t="s">
         <v>7</v>
@@ -1717,19 +1723,19 @@
         <v>32</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>129</v>
+        <v>170</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>181</v>
+        <v>150</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>130</v>
+        <v>171</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>202</v>
+        <v>172</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>7</v>
@@ -1740,42 +1746,42 @@
         <v>33</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>131</v>
+        <v>173</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>182</v>
+        <v>150</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>46</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>132</v>
+        <v>174</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>192</v>
+        <v>175</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>203</v>
+        <v>176</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>182</v>
+        <v>150</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E36" s="6" t="s">
-        <v>204</v>
+      <c r="E36" s="8" t="s">
+        <v>177</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>205</v>
+        <v>167</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>7</v>
@@ -1786,42 +1792,42 @@
         <v>35</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>206</v>
+        <v>178</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>182</v>
+        <v>151</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>207</v>
+        <v>157</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>208</v>
+        <v>179</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>209</v>
+        <v>125</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>182</v>
+        <v>151</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>210</v>
+        <v>53</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>126</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>200</v>
+        <v>162</v>
       </c>
       <c r="G38" s="1" t="s">
         <v>7</v>
@@ -1832,19 +1838,19 @@
         <v>37</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>211</v>
+        <v>181</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>183</v>
+        <v>152</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>189</v>
+        <v>127</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>212</v>
+        <v>160</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>7</v>
@@ -1855,22 +1861,22 @@
         <v>38</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>183</v>
+        <v>152</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>194</v>
+        <v>160</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1878,20 +1884,22 @@
         <v>39</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>58</v>
+        <v>183</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>184</v>
+        <v>153</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>58</v>
+        <v>182</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="F41" s="1"/>
+        <v>214</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>166</v>
+      </c>
       <c r="G41" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1899,20 +1907,22 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>136</v>
+        <v>184</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>184</v>
+        <v>153</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>58</v>
+        <v>182</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="F42" s="1"/>
+        <v>188</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>168</v>
+      </c>
       <c r="G42" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1920,18 +1930,20 @@
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>184</v>
+        <v>153</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>58</v>
+        <v>182</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="F43" s="1"/>
+        <v>189</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>190</v>
+      </c>
       <c r="G43" s="1" t="s">
         <v>9</v>
       </c>
@@ -1941,41 +1953,45 @@
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>140</v>
+        <v>185</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>185</v>
+        <v>153</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>63</v>
+        <v>182</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="F44" s="1"/>
+        <v>191</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>190</v>
+      </c>
       <c r="G44" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>142</v>
+        <v>186</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>185</v>
+        <v>153</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>63</v>
+        <v>182</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="F45" s="1"/>
+        <v>192</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>193</v>
+      </c>
       <c r="G45" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1983,18 +1999,20 @@
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>185</v>
+        <v>62</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>63</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="F46" s="1"/>
+        <v>213</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>167</v>
+      </c>
       <c r="G46" s="1" t="s">
         <v>9</v>
       </c>
@@ -2004,39 +2022,43 @@
         <v>47</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>146</v>
+        <v>194</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>185</v>
+        <v>72</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="F47" s="1"/>
+        <v>134</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>160</v>
+      </c>
       <c r="G47" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>148</v>
+        <v>195</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="F48" s="1"/>
+        <v>212</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="G48" s="1" t="s">
         <v>9</v>
       </c>
@@ -2046,18 +2068,20 @@
         <v>49</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>150</v>
+        <v>196</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="F49" s="1"/>
+        <v>131</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>162</v>
+      </c>
       <c r="G49" s="1" t="s">
         <v>7</v>
       </c>
@@ -2067,20 +2091,22 @@
         <v>50</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>152</v>
+        <v>197</v>
       </c>
       <c r="C50" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D50" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="E50" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="F50" s="1"/>
+        <v>133</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>132</v>
+      </c>
       <c r="G50" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2088,18 +2114,20 @@
         <v>51</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>154</v>
+        <v>201</v>
       </c>
       <c r="C51" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D51" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D51" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="E51" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="F51" s="1"/>
+        <v>198</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>199</v>
+      </c>
       <c r="G51" s="1" t="s">
         <v>9</v>
       </c>
@@ -2109,41 +2137,45 @@
         <v>52</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>156</v>
+        <v>202</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="F52" s="1"/>
+        <v>203</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>200</v>
+      </c>
       <c r="G52" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>158</v>
+        <v>207</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="F53" s="1"/>
+        <v>206</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>190</v>
+      </c>
       <c r="G53" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2151,20 +2183,22 @@
         <v>55</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>77</v>
+        <v>135</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>76</v>
+        <v>205</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>77</v>
+        <v>136</v>
       </c>
       <c r="E54" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="F54" s="1"/>
       <c r="G54" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2172,18 +2206,20 @@
         <v>56</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>161</v>
+        <v>138</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>78</v>
+        <v>205</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>79</v>
+        <v>136</v>
       </c>
       <c r="E55" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="F55" s="1"/>
       <c r="G55" s="1" t="s">
         <v>9</v>
       </c>
@@ -2193,20 +2229,22 @@
         <v>57</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>80</v>
+        <v>205</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="F56" s="1"/>
+        <v>142</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>190</v>
+      </c>
       <c r="G56" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2214,103 +2252,67 @@
         <v>59</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>80</v>
+        <v>205</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="F57" s="1"/>
+        <v>144</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>190</v>
+      </c>
       <c r="G57" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>168</v>
+        <v>210</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>69</v>
+        <v>215</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>169</v>
+        <v>76</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="F58" s="1"/>
+        <v>211</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>76</v>
+      </c>
       <c r="G58" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>171</v>
+        <v>208</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>69</v>
+        <v>215</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>169</v>
+        <v>77</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="F59" s="1"/>
+        <v>209</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>77</v>
+      </c>
       <c r="G59" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A60" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E60" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="F60" s="1"/>
-      <c r="G60" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A61" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="F61" s="1"/>
-      <c r="G61" s="1" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>